<commit_message>
build: sync from ULLL/UMKK/shared by metramak
</commit_message>
<xml_diff>
--- a/ULLL/Plugins/# Docs/TopSky Documentation/Developer/TopSky_Developer_Guide_Settings.xlsx
+++ b/ULLL/Plugins/# Docs/TopSky Documentation/Developer/TopSky_Developer_Guide_Settings.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Juha\Documents\Office Files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A6C412C-E0A6-4130-AABA-20EBF9B17743}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE00DD0E-6EB2-43B5-B5EE-9B569D508039}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10605" yWindow="1680" windowWidth="21585" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4440" yWindow="2865" windowWidth="21585" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TopSky 2.6" sheetId="1" r:id="rId1"/>
@@ -7421,9 +7421,6 @@
     <t>NOTAM data source</t>
   </si>
   <si>
-    <t>0 (custom, use below settings to define) or 1 (VATSIM Radar)</t>
-  </si>
-  <si>
     <t>https://notams.aim.faa.gov/nat.html</t>
   </si>
   <si>
@@ -8320,6 +8317,9 @@
   </si>
   <si>
     <t>No "R" flags for aircraft with no predicted path points above this level</t>
+  </si>
+  <si>
+    <t>0 (custom, use below settings to define - to override the plugin-provided list of location codes, define the whole URL in HTTP_NOTAM_Server and leave the page prefix and suffix settings empty) or 1 (VATSIM Radar - the server and page settings below are not used)</t>
   </si>
 </sst>
 </file>
@@ -12211,13 +12211,13 @@
         <v>1261</v>
       </c>
       <c r="B10" t="s">
-        <v>2712</v>
+        <v>2711</v>
       </c>
       <c r="C10" t="s">
         <v>721</v>
       </c>
       <c r="D10" t="s">
-        <v>2470</v>
+        <v>2469</v>
       </c>
       <c r="E10" s="4" t="s">
         <v>721</v>
@@ -12431,7 +12431,7 @@
         <v>1031</v>
       </c>
       <c r="B22" t="s">
-        <v>2544</v>
+        <v>2543</v>
       </c>
       <c r="C22" t="s">
         <v>721</v>
@@ -12526,10 +12526,10 @@
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>2753</v>
+      </c>
+      <c r="B26" t="s">
         <v>2754</v>
-      </c>
-      <c r="B26" t="s">
-        <v>2755</v>
       </c>
       <c r="C26" t="s">
         <v>721</v>
@@ -12864,7 +12864,7 @@
         <v>1581</v>
       </c>
       <c r="B44" t="s">
-        <v>2663</v>
+        <v>2662</v>
       </c>
       <c r="C44" t="s">
         <v>721</v>
@@ -13079,10 +13079,10 @@
     </row>
     <row r="55" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
       <c r="B55" t="s">
-        <v>2569</v>
+        <v>2568</v>
       </c>
       <c r="C55" t="s">
         <v>721</v>
@@ -13105,10 +13105,10 @@
     </row>
     <row r="56" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
       <c r="B56" t="s">
-        <v>2570</v>
+        <v>2569</v>
       </c>
       <c r="C56" t="s">
         <v>721</v>
@@ -13485,7 +13485,7 @@
         <v>238</v>
       </c>
       <c r="B73" t="s">
-        <v>2753</v>
+        <v>2752</v>
       </c>
       <c r="C73" t="s">
         <v>721</v>
@@ -14005,16 +14005,16 @@
     </row>
     <row r="98" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
+        <v>2668</v>
+      </c>
+      <c r="B98" t="s">
         <v>2669</v>
       </c>
-      <c r="B98" t="s">
-        <v>2670</v>
-      </c>
       <c r="C98" t="s">
         <v>721</v>
       </c>
       <c r="D98" s="6" t="s">
-        <v>2581</v>
+        <v>2580</v>
       </c>
       <c r="E98" s="4" t="s">
         <v>721</v>
@@ -14028,10 +14028,10 @@
     </row>
     <row r="99" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
+        <v>2670</v>
+      </c>
+      <c r="B99" t="s">
         <v>2671</v>
-      </c>
-      <c r="B99" t="s">
-        <v>2672</v>
       </c>
       <c r="C99" t="s">
         <v>721</v>
@@ -14043,7 +14043,7 @@
         <v>173</v>
       </c>
       <c r="F99" s="4" t="s">
-        <v>2673</v>
+        <v>2672</v>
       </c>
       <c r="H99" s="2">
         <v>50</v>
@@ -14054,10 +14054,10 @@
     </row>
     <row r="100" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>2703</v>
+        <v>2702</v>
       </c>
       <c r="B100" t="s">
-        <v>2674</v>
+        <v>2673</v>
       </c>
       <c r="C100" t="s">
         <v>721</v>
@@ -14080,10 +14080,10 @@
     </row>
     <row r="101" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
+        <v>2704</v>
+      </c>
+      <c r="B101" t="s">
         <v>2705</v>
-      </c>
-      <c r="B101" t="s">
-        <v>2706</v>
       </c>
       <c r="C101" t="s">
         <v>721</v>
@@ -14118,10 +14118,10 @@
         <v>129</v>
       </c>
       <c r="H103" s="2" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
       <c r="I103" s="2" t="s">
-        <v>2545</v>
+        <v>2544</v>
       </c>
     </row>
     <row r="104" spans="1:9" x14ac:dyDescent="0.25">
@@ -14646,7 +14646,7 @@
     </row>
     <row r="130" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
       <c r="B130" t="s">
         <v>556</v>
@@ -14661,7 +14661,7 @@
         <v>58</v>
       </c>
       <c r="I130" s="2" t="s">
-        <v>2565</v>
+        <v>2564</v>
       </c>
     </row>
     <row r="131" spans="1:9" x14ac:dyDescent="0.25">
@@ -14766,7 +14766,7 @@
     </row>
     <row r="136" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>2713</v>
+        <v>2712</v>
       </c>
       <c r="B136" t="s">
         <v>556</v>
@@ -14781,12 +14781,12 @@
         <v>74</v>
       </c>
       <c r="I136" s="2" t="s">
-        <v>2718</v>
+        <v>2717</v>
       </c>
     </row>
     <row r="137" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>2714</v>
+        <v>2713</v>
       </c>
       <c r="B137" t="s">
         <v>556</v>
@@ -14801,12 +14801,12 @@
         <v>1622</v>
       </c>
       <c r="I137" s="2" t="s">
-        <v>2719</v>
+        <v>2718</v>
       </c>
     </row>
     <row r="138" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>2715</v>
+        <v>2714</v>
       </c>
       <c r="B138" t="s">
         <v>556</v>
@@ -14821,12 +14821,12 @@
         <v>1622</v>
       </c>
       <c r="I138" s="2" t="s">
-        <v>2720</v>
+        <v>2719</v>
       </c>
     </row>
     <row r="139" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>2716</v>
+        <v>2715</v>
       </c>
       <c r="B139" t="s">
         <v>556</v>
@@ -14838,15 +14838,15 @@
         <v>129</v>
       </c>
       <c r="H139" s="2" t="s">
-        <v>2721</v>
+        <v>2720</v>
       </c>
       <c r="I139" s="2" t="s">
-        <v>2721</v>
+        <v>2720</v>
       </c>
     </row>
     <row r="140" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>2717</v>
+        <v>2716</v>
       </c>
       <c r="B140" t="s">
         <v>556</v>
@@ -14858,10 +14858,10 @@
         <v>129</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>2722</v>
+        <v>2721</v>
       </c>
       <c r="I140" s="2" t="s">
-        <v>2722</v>
+        <v>2721</v>
       </c>
     </row>
     <row r="141" spans="1:9" x14ac:dyDescent="0.25">
@@ -15166,7 +15166,7 @@
         <v>965</v>
       </c>
       <c r="I156" s="2" t="s">
-        <v>2554</v>
+        <v>2553</v>
       </c>
     </row>
     <row r="157" spans="1:9" x14ac:dyDescent="0.25">
@@ -15206,7 +15206,7 @@
         <v>968</v>
       </c>
       <c r="I158" s="2" t="s">
-        <v>2555</v>
+        <v>2554</v>
       </c>
     </row>
     <row r="159" spans="1:9" x14ac:dyDescent="0.25">
@@ -15516,7 +15516,7 @@
     </row>
     <row r="175" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
       <c r="B175" t="s">
         <v>556</v>
@@ -15531,12 +15531,12 @@
         <v>55</v>
       </c>
       <c r="I175" s="2" t="s">
-        <v>2549</v>
+        <v>2548</v>
       </c>
     </row>
     <row r="176" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
       <c r="B176" t="s">
         <v>556</v>
@@ -15551,12 +15551,12 @@
         <v>68</v>
       </c>
       <c r="I176" s="2" t="s">
-        <v>2547</v>
+        <v>2546</v>
       </c>
     </row>
     <row r="177" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
       <c r="B177" t="s">
         <v>556</v>
@@ -15571,12 +15571,12 @@
         <v>55</v>
       </c>
       <c r="I177" s="2" t="s">
-        <v>2551</v>
+        <v>2550</v>
       </c>
     </row>
     <row r="178" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
       <c r="B178" t="s">
         <v>556</v>
@@ -15591,7 +15591,7 @@
         <v>55</v>
       </c>
       <c r="I178" s="2" t="s">
-        <v>2560</v>
+        <v>2559</v>
       </c>
     </row>
     <row r="179" spans="1:9" x14ac:dyDescent="0.25">
@@ -15711,7 +15711,7 @@
         <v>637</v>
       </c>
       <c r="I184" s="2" t="s">
-        <v>2556</v>
+        <v>2555</v>
       </c>
     </row>
     <row r="185" spans="1:9" x14ac:dyDescent="0.25">
@@ -16022,7 +16022,7 @@
         <v>129</v>
       </c>
       <c r="I200" s="2" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="201" spans="1:9" x14ac:dyDescent="0.25">
@@ -16039,7 +16039,7 @@
         <v>129</v>
       </c>
       <c r="I201" s="2" t="s">
-        <v>2552</v>
+        <v>2551</v>
       </c>
     </row>
     <row r="202" spans="1:9" x14ac:dyDescent="0.25">
@@ -16199,7 +16199,7 @@
         <v>1628</v>
       </c>
       <c r="I209" s="2" t="s">
-        <v>2557</v>
+        <v>2556</v>
       </c>
     </row>
     <row r="210" spans="1:9" x14ac:dyDescent="0.25">
@@ -16658,7 +16658,7 @@
     </row>
     <row r="233" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
       <c r="B233" t="s">
         <v>556</v>
@@ -17055,12 +17055,12 @@
         <v>129</v>
       </c>
       <c r="I253" s="2" t="s">
-        <v>2553</v>
+        <v>2552</v>
       </c>
     </row>
     <row r="254" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A254" t="s">
-        <v>2723</v>
+        <v>2722</v>
       </c>
       <c r="B254" t="s">
         <v>556</v>
@@ -17072,15 +17072,15 @@
         <v>129</v>
       </c>
       <c r="H254" s="2" t="s">
-        <v>2727</v>
+        <v>2726</v>
       </c>
       <c r="I254" s="2" t="s">
-        <v>2727</v>
+        <v>2726</v>
       </c>
     </row>
     <row r="255" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A255" t="s">
-        <v>2724</v>
+        <v>2723</v>
       </c>
       <c r="B255" t="s">
         <v>556</v>
@@ -17092,15 +17092,15 @@
         <v>129</v>
       </c>
       <c r="H255" s="2" t="s">
-        <v>2728</v>
+        <v>2727</v>
       </c>
       <c r="I255" s="2" t="s">
-        <v>2728</v>
+        <v>2727</v>
       </c>
     </row>
     <row r="256" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A256" t="s">
-        <v>2725</v>
+        <v>2724</v>
       </c>
       <c r="B256" t="s">
         <v>556</v>
@@ -17112,15 +17112,15 @@
         <v>129</v>
       </c>
       <c r="H256" s="2" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
       <c r="I256" s="2" t="s">
-        <v>2729</v>
+        <v>2728</v>
       </c>
     </row>
     <row r="257" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A257" t="s">
-        <v>2726</v>
+        <v>2725</v>
       </c>
       <c r="B257" t="s">
         <v>556</v>
@@ -17132,10 +17132,10 @@
         <v>129</v>
       </c>
       <c r="H257" s="2" t="s">
-        <v>2730</v>
+        <v>2729</v>
       </c>
       <c r="I257" s="2" t="s">
-        <v>2730</v>
+        <v>2729</v>
       </c>
     </row>
     <row r="258" spans="1:9" x14ac:dyDescent="0.25">
@@ -17672,7 +17672,7 @@
         <v>73</v>
       </c>
       <c r="I284" s="2" t="s">
-        <v>2558</v>
+        <v>2557</v>
       </c>
     </row>
     <row r="286" spans="1:9" x14ac:dyDescent="0.25">
@@ -17843,16 +17843,16 @@
     </row>
     <row r="294" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A294" t="s">
+        <v>2473</v>
+      </c>
+      <c r="B294" t="s">
         <v>2474</v>
       </c>
-      <c r="B294" t="s">
-        <v>2475</v>
-      </c>
       <c r="C294" t="s">
         <v>721</v>
       </c>
       <c r="D294" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="E294" s="4" t="s">
         <v>721</v>
@@ -17866,16 +17866,16 @@
     </row>
     <row r="295" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A295" t="s">
+        <v>2470</v>
+      </c>
+      <c r="B295" t="s">
         <v>2471</v>
       </c>
-      <c r="B295" t="s">
+      <c r="C295" t="s">
+        <v>721</v>
+      </c>
+      <c r="D295" t="s">
         <v>2472</v>
-      </c>
-      <c r="C295" t="s">
-        <v>721</v>
-      </c>
-      <c r="D295" t="s">
-        <v>2473</v>
       </c>
       <c r="E295" s="4" t="s">
         <v>721</v>
@@ -17889,16 +17889,16 @@
     </row>
     <row r="296" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A296" t="s">
+        <v>2475</v>
+      </c>
+      <c r="B296" t="s">
         <v>2476</v>
       </c>
-      <c r="B296" t="s">
-        <v>2477</v>
-      </c>
       <c r="C296" t="s">
         <v>721</v>
       </c>
       <c r="D296" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="E296" s="4" t="s">
         <v>721</v>
@@ -17912,16 +17912,16 @@
     </row>
     <row r="297" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A297" t="s">
+        <v>2477</v>
+      </c>
+      <c r="B297" t="s">
         <v>2478</v>
       </c>
-      <c r="B297" t="s">
-        <v>2479</v>
-      </c>
       <c r="C297" t="s">
         <v>721</v>
       </c>
       <c r="D297" t="s">
-        <v>2473</v>
+        <v>2472</v>
       </c>
       <c r="E297" s="4" t="s">
         <v>721</v>
@@ -17935,10 +17935,10 @@
     </row>
     <row r="298" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A298" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
       <c r="B298" t="s">
-        <v>2483</v>
+        <v>2482</v>
       </c>
       <c r="C298" t="s">
         <v>721</v>
@@ -17958,10 +17958,10 @@
     </row>
     <row r="299" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A299" t="s">
+        <v>2480</v>
+      </c>
+      <c r="B299" t="s">
         <v>2481</v>
-      </c>
-      <c r="B299" t="s">
-        <v>2482</v>
       </c>
       <c r="C299" t="s">
         <v>721</v>
@@ -18153,16 +18153,16 @@
     </row>
     <row r="308" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A308" t="s">
+        <v>2739</v>
+      </c>
+      <c r="B308" t="s">
         <v>2740</v>
       </c>
-      <c r="B308" t="s">
-        <v>2741</v>
-      </c>
       <c r="C308" t="s">
         <v>721</v>
       </c>
       <c r="D308" t="s">
-        <v>2751</v>
+        <v>2750</v>
       </c>
       <c r="E308" s="4" t="s">
         <v>721</v>
@@ -18539,10 +18539,10 @@
         <v>130</v>
       </c>
       <c r="H324" s="2" t="s">
-        <v>2742</v>
+        <v>2741</v>
       </c>
       <c r="I324" s="2" t="s">
-        <v>2742</v>
+        <v>2741</v>
       </c>
     </row>
     <row r="325" spans="1:9" x14ac:dyDescent="0.25">
@@ -18559,10 +18559,10 @@
         <v>130</v>
       </c>
       <c r="H325" s="2" t="s">
-        <v>2743</v>
+        <v>2742</v>
       </c>
       <c r="I325" s="2" t="s">
-        <v>2743</v>
+        <v>2742</v>
       </c>
     </row>
     <row r="326" spans="1:9" x14ac:dyDescent="0.25">
@@ -18587,10 +18587,10 @@
     </row>
     <row r="327" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A327" t="s">
+        <v>2733</v>
+      </c>
+      <c r="B327" t="s">
         <v>2734</v>
-      </c>
-      <c r="B327" t="s">
-        <v>2735</v>
       </c>
       <c r="C327" t="s">
         <v>721</v>
@@ -18599,10 +18599,10 @@
         <v>130</v>
       </c>
       <c r="H327" s="2" t="s">
-        <v>2738</v>
+        <v>2737</v>
       </c>
       <c r="I327" s="2" t="s">
-        <v>2738</v>
+        <v>2737</v>
       </c>
     </row>
     <row r="328" spans="1:9" x14ac:dyDescent="0.25">
@@ -18619,10 +18619,10 @@
         <v>130</v>
       </c>
       <c r="H328" s="2" t="s">
-        <v>2745</v>
+        <v>2744</v>
       </c>
       <c r="I328" s="2" t="s">
-        <v>2745</v>
+        <v>2744</v>
       </c>
     </row>
     <row r="329" spans="1:9" x14ac:dyDescent="0.25">
@@ -18639,10 +18639,10 @@
         <v>130</v>
       </c>
       <c r="H329" s="2" t="s">
-        <v>2744</v>
+        <v>2743</v>
       </c>
       <c r="I329" s="2" t="s">
-        <v>2744</v>
+        <v>2743</v>
       </c>
     </row>
     <row r="330" spans="1:9" x14ac:dyDescent="0.25">
@@ -18659,10 +18659,10 @@
         <v>130</v>
       </c>
       <c r="H330" s="2" t="s">
-        <v>2746</v>
+        <v>2745</v>
       </c>
       <c r="I330" s="2" t="s">
-        <v>2746</v>
+        <v>2745</v>
       </c>
     </row>
     <row r="331" spans="1:9" x14ac:dyDescent="0.25">
@@ -18679,10 +18679,10 @@
         <v>130</v>
       </c>
       <c r="H331" s="2" t="s">
-        <v>2747</v>
+        <v>2746</v>
       </c>
       <c r="I331" s="2" t="s">
-        <v>2747</v>
+        <v>2746</v>
       </c>
     </row>
     <row r="332" spans="1:9" x14ac:dyDescent="0.25">
@@ -18699,15 +18699,15 @@
         <v>130</v>
       </c>
       <c r="H332" s="2" t="s">
-        <v>2748</v>
+        <v>2747</v>
       </c>
       <c r="I332" s="2" t="s">
-        <v>2748</v>
+        <v>2747</v>
       </c>
     </row>
     <row r="333" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A333" t="s">
-        <v>2736</v>
+        <v>2735</v>
       </c>
       <c r="B333" t="s">
         <v>1325</v>
@@ -18719,10 +18719,10 @@
         <v>130</v>
       </c>
       <c r="H333" s="2" t="s">
-        <v>2739</v>
+        <v>2738</v>
       </c>
       <c r="I333" s="2" t="s">
-        <v>2739</v>
+        <v>2738</v>
       </c>
     </row>
     <row r="334" spans="1:9" x14ac:dyDescent="0.25">
@@ -18739,10 +18739,10 @@
         <v>130</v>
       </c>
       <c r="H334" s="2" t="s">
-        <v>2749</v>
+        <v>2748</v>
       </c>
       <c r="I334" s="2" t="s">
-        <v>2749</v>
+        <v>2748</v>
       </c>
     </row>
     <row r="335" spans="1:9" x14ac:dyDescent="0.25">
@@ -18759,10 +18759,10 @@
         <v>130</v>
       </c>
       <c r="H335" s="2" t="s">
-        <v>2750</v>
+        <v>2749</v>
       </c>
       <c r="I335" s="2" t="s">
-        <v>2750</v>
+        <v>2749</v>
       </c>
     </row>
     <row r="336" spans="1:9" x14ac:dyDescent="0.25">
@@ -18925,7 +18925,7 @@
         <v>1431</v>
       </c>
       <c r="B344" t="s">
-        <v>2664</v>
+        <v>2663</v>
       </c>
       <c r="C344" t="s">
         <v>721</v>
@@ -19633,10 +19633,10 @@
     </row>
     <row r="379" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A379" t="s">
+        <v>2507</v>
+      </c>
+      <c r="B379" t="s">
         <v>2508</v>
-      </c>
-      <c r="B379" t="s">
-        <v>2509</v>
       </c>
       <c r="C379" t="s">
         <v>721</v>
@@ -19653,16 +19653,16 @@
     </row>
     <row r="380" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A380" t="s">
+        <v>2509</v>
+      </c>
+      <c r="B380" t="s">
         <v>2510</v>
       </c>
-      <c r="B380" t="s">
+      <c r="C380" t="s">
+        <v>721</v>
+      </c>
+      <c r="D380" t="s">
         <v>2511</v>
-      </c>
-      <c r="C380" t="s">
-        <v>721</v>
-      </c>
-      <c r="D380" t="s">
-        <v>2512</v>
       </c>
       <c r="E380" s="4" t="s">
         <v>721</v>
@@ -19676,16 +19676,16 @@
     </row>
     <row r="381" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A381" t="s">
+        <v>2512</v>
+      </c>
+      <c r="B381" t="s">
         <v>2513</v>
       </c>
-      <c r="B381" t="s">
+      <c r="C381" t="s">
+        <v>721</v>
+      </c>
+      <c r="D381" t="s">
         <v>2514</v>
-      </c>
-      <c r="C381" t="s">
-        <v>721</v>
-      </c>
-      <c r="D381" t="s">
-        <v>2515</v>
       </c>
       <c r="E381" s="4" t="s">
         <v>721</v>
@@ -19699,16 +19699,16 @@
     </row>
     <row r="382" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A382" t="s">
+        <v>2515</v>
+      </c>
+      <c r="B382" t="s">
         <v>2516</v>
       </c>
-      <c r="B382" t="s">
+      <c r="C382" t="s">
+        <v>721</v>
+      </c>
+      <c r="D382" t="s">
         <v>2517</v>
-      </c>
-      <c r="C382" t="s">
-        <v>721</v>
-      </c>
-      <c r="D382" t="s">
-        <v>2518</v>
       </c>
       <c r="E382" s="4" t="s">
         <v>721</v>
@@ -19722,10 +19722,10 @@
     </row>
     <row r="383" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A383" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
       <c r="B383" t="s">
-        <v>2542</v>
+        <v>2541</v>
       </c>
       <c r="C383" t="s">
         <v>721</v>
@@ -19742,10 +19742,10 @@
     </row>
     <row r="384" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A384" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
       <c r="B384" t="s">
-        <v>2541</v>
+        <v>2540</v>
       </c>
       <c r="C384" t="s">
         <v>721</v>
@@ -19762,10 +19762,10 @@
     </row>
     <row r="385" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A385" t="s">
+        <v>2520</v>
+      </c>
+      <c r="B385" t="s">
         <v>2521</v>
-      </c>
-      <c r="B385" t="s">
-        <v>2522</v>
       </c>
       <c r="C385" t="s">
         <v>721</v>
@@ -19788,10 +19788,10 @@
     </row>
     <row r="386" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A386" t="s">
+        <v>2538</v>
+      </c>
+      <c r="B386" t="s">
         <v>2539</v>
-      </c>
-      <c r="B386" t="s">
-        <v>2540</v>
       </c>
       <c r="C386" t="s">
         <v>721</v>
@@ -19814,10 +19814,10 @@
     </row>
     <row r="387" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A387" t="s">
+        <v>2522</v>
+      </c>
+      <c r="B387" t="s">
         <v>2523</v>
-      </c>
-      <c r="B387" t="s">
-        <v>2524</v>
       </c>
       <c r="C387" t="s">
         <v>721</v>
@@ -19840,10 +19840,10 @@
     </row>
     <row r="388" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A388" t="s">
+        <v>2524</v>
+      </c>
+      <c r="B388" t="s">
         <v>2525</v>
-      </c>
-      <c r="B388" t="s">
-        <v>2526</v>
       </c>
       <c r="C388" t="s">
         <v>721</v>
@@ -20496,16 +20496,16 @@
     </row>
     <row r="419" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A419" t="s">
+        <v>2486</v>
+      </c>
+      <c r="B419" t="s">
         <v>2487</v>
       </c>
-      <c r="B419" t="s">
-        <v>2488</v>
-      </c>
       <c r="C419" t="s">
         <v>721</v>
       </c>
       <c r="D419" t="s">
-        <v>2490</v>
+        <v>2489</v>
       </c>
       <c r="E419" s="4" t="s">
         <v>721</v>
@@ -20849,10 +20849,10 @@
         <v>130</v>
       </c>
       <c r="H443" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
       <c r="I443" t="s">
-        <v>2458</v>
+        <v>2457</v>
       </c>
     </row>
     <row r="444" spans="1:9" x14ac:dyDescent="0.25">
@@ -21073,16 +21073,16 @@
         <v>721</v>
       </c>
       <c r="D455" t="s">
-        <v>2457</v>
+        <v>2755</v>
       </c>
       <c r="E455" s="4" t="s">
         <v>721</v>
       </c>
       <c r="H455" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I455" s="2">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="456" spans="1:9" x14ac:dyDescent="0.25">
@@ -21214,13 +21214,13 @@
         <v>2454</v>
       </c>
       <c r="B465" t="s">
-        <v>2489</v>
+        <v>2488</v>
       </c>
       <c r="C465" t="s">
         <v>721</v>
       </c>
       <c r="D465" t="s">
-        <v>2486</v>
+        <v>2485</v>
       </c>
       <c r="E465" s="4" t="s">
         <v>721</v>
@@ -22007,7 +22007,7 @@
         <v>130</v>
       </c>
       <c r="I502" s="2" t="s">
-        <v>2752</v>
+        <v>2751</v>
       </c>
     </row>
     <row r="503" spans="1:9" x14ac:dyDescent="0.25">
@@ -23131,7 +23131,7 @@
     </row>
     <row r="561" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A561" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
       <c r="B561" t="s">
         <v>2044</v>
@@ -23272,7 +23272,7 @@
     </row>
     <row r="568" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A568" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="B568" t="s">
         <v>2044</v>
@@ -23519,10 +23519,10 @@
     </row>
     <row r="582" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A582" t="s">
+        <v>2490</v>
+      </c>
+      <c r="B582" t="s">
         <v>2491</v>
-      </c>
-      <c r="B582" t="s">
-        <v>2492</v>
       </c>
       <c r="C582" t="s">
         <v>721</v>
@@ -23545,10 +23545,10 @@
     </row>
     <row r="583" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A583" t="s">
+        <v>2492</v>
+      </c>
+      <c r="B583" t="s">
         <v>2493</v>
-      </c>
-      <c r="B583" t="s">
-        <v>2494</v>
       </c>
       <c r="C583" t="s">
         <v>721</v>
@@ -23565,16 +23565,16 @@
     </row>
     <row r="584" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A584" t="s">
+        <v>2494</v>
+      </c>
+      <c r="B584" t="s">
         <v>2495</v>
       </c>
-      <c r="B584" t="s">
+      <c r="C584" t="s">
+        <v>721</v>
+      </c>
+      <c r="D584" s="6" t="s">
         <v>2496</v>
-      </c>
-      <c r="C584" t="s">
-        <v>721</v>
-      </c>
-      <c r="D584" s="6" t="s">
-        <v>2497</v>
       </c>
       <c r="E584" s="4" t="s">
         <v>721</v>
@@ -23588,16 +23588,16 @@
     </row>
     <row r="585" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A585" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
       <c r="B585" t="s">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="C585" t="s">
         <v>721</v>
       </c>
       <c r="D585" s="6" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="E585" s="4" t="s">
         <v>721</v>
@@ -23611,16 +23611,16 @@
     </row>
     <row r="586" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A586" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
       <c r="B586" t="s">
-        <v>2504</v>
+        <v>2503</v>
       </c>
       <c r="C586" t="s">
         <v>721</v>
       </c>
       <c r="D586" s="6" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="E586" s="4" t="s">
         <v>721</v>
@@ -23634,16 +23634,16 @@
     </row>
     <row r="587" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A587" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
       <c r="B587" t="s">
-        <v>2505</v>
+        <v>2504</v>
       </c>
       <c r="C587" t="s">
         <v>721</v>
       </c>
       <c r="D587" s="6" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="E587" s="4" t="s">
         <v>721</v>
@@ -23657,16 +23657,16 @@
     </row>
     <row r="588" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A588" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
       <c r="B588" t="s">
-        <v>2506</v>
+        <v>2505</v>
       </c>
       <c r="C588" t="s">
         <v>721</v>
       </c>
       <c r="D588" s="6" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="E588" s="4" t="s">
         <v>721</v>
@@ -23680,16 +23680,16 @@
     </row>
     <row r="589" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A589" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="B589" t="s">
-        <v>2507</v>
+        <v>2506</v>
       </c>
       <c r="C589" t="s">
         <v>721</v>
       </c>
       <c r="D589" s="6" t="s">
-        <v>2497</v>
+        <v>2496</v>
       </c>
       <c r="E589" s="4" t="s">
         <v>721</v>
@@ -24148,10 +24148,10 @@
     </row>
     <row r="610" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A610" t="s">
+        <v>2570</v>
+      </c>
+      <c r="B610" t="s">
         <v>2571</v>
-      </c>
-      <c r="B610" t="s">
-        <v>2572</v>
       </c>
       <c r="C610" t="s">
         <v>721</v>
@@ -24344,7 +24344,7 @@
         <v>721</v>
       </c>
       <c r="D618" s="6" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
       <c r="E618" s="4" t="s">
         <v>721</v>
@@ -24430,7 +24430,7 @@
         <v>721</v>
       </c>
       <c r="D622" s="6" t="s">
-        <v>2566</v>
+        <v>2565</v>
       </c>
       <c r="E622" s="4" t="s">
         <v>721</v>
@@ -25825,7 +25825,7 @@
         <v>721</v>
       </c>
       <c r="D690" t="s">
-        <v>2707</v>
+        <v>2706</v>
       </c>
       <c r="E690" s="4" t="s">
         <v>721</v>
@@ -26119,7 +26119,7 @@
         <v>721</v>
       </c>
       <c r="D703" t="s">
-        <v>2468</v>
+        <v>2467</v>
       </c>
       <c r="E703" s="4" t="s">
         <v>721</v>
@@ -26208,10 +26208,10 @@
     </row>
     <row r="708" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A708" t="s">
+        <v>2483</v>
+      </c>
+      <c r="B708" t="s">
         <v>2484</v>
-      </c>
-      <c r="B708" t="s">
-        <v>2485</v>
       </c>
       <c r="D708" t="s">
         <v>128</v>
@@ -26225,13 +26225,13 @@
     </row>
     <row r="709" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A709" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
       <c r="B709" t="s">
-        <v>2467</v>
+        <v>2466</v>
       </c>
       <c r="D709" t="s">
-        <v>2469</v>
+        <v>2468</v>
       </c>
       <c r="E709" s="4" t="s">
         <v>721</v>
@@ -26242,7 +26242,7 @@
         <v>166</v>
       </c>
       <c r="B710" t="s">
-        <v>2466</v>
+        <v>2465</v>
       </c>
       <c r="C710" t="s">
         <v>721</v>
@@ -26698,7 +26698,7 @@
         <v>721</v>
       </c>
       <c r="D730" t="s">
-        <v>2708</v>
+        <v>2707</v>
       </c>
       <c r="E730" s="4" t="s">
         <v>721</v>
@@ -30542,10 +30542,10 @@
     </row>
     <row r="898" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A898" t="s">
-        <v>2733</v>
+        <v>2732</v>
       </c>
       <c r="B898" t="s">
-        <v>2737</v>
+        <v>2736</v>
       </c>
       <c r="C898" t="s">
         <v>721</v>
@@ -31060,10 +31060,10 @@
     </row>
     <row r="920" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A920" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
       <c r="B920" t="s">
-        <v>2533</v>
+        <v>2532</v>
       </c>
       <c r="C920" t="s">
         <v>721</v>
@@ -31080,10 +31080,10 @@
     </row>
     <row r="921" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A921" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
       <c r="B921" t="s">
-        <v>2537</v>
+        <v>2536</v>
       </c>
       <c r="C921" t="s">
         <v>721</v>
@@ -31106,10 +31106,10 @@
     </row>
     <row r="922" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A922" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
       <c r="B922" t="s">
-        <v>2534</v>
+        <v>2533</v>
       </c>
       <c r="C922" t="s">
         <v>721</v>
@@ -31129,10 +31129,10 @@
     </row>
     <row r="923" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A923" t="s">
-        <v>2530</v>
+        <v>2529</v>
       </c>
       <c r="B923" t="s">
-        <v>2536</v>
+        <v>2535</v>
       </c>
       <c r="C923" t="s">
         <v>721</v>
@@ -31149,10 +31149,10 @@
     </row>
     <row r="924" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A924" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
       <c r="B924" t="s">
-        <v>2538</v>
+        <v>2537</v>
       </c>
       <c r="C924" t="s">
         <v>721</v>
@@ -31175,10 +31175,10 @@
     </row>
     <row r="925" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A925" t="s">
-        <v>2532</v>
+        <v>2531</v>
       </c>
       <c r="B925" t="s">
-        <v>2535</v>
+        <v>2534</v>
       </c>
       <c r="C925" t="s">
         <v>721</v>
@@ -31824,16 +31824,16 @@
     </row>
     <row r="954" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A954" t="s">
+        <v>2708</v>
+      </c>
+      <c r="B954" t="s">
         <v>2709</v>
       </c>
-      <c r="B954" t="s">
+      <c r="C954" t="s">
+        <v>721</v>
+      </c>
+      <c r="D954" t="s">
         <v>2710</v>
-      </c>
-      <c r="C954" t="s">
-        <v>721</v>
-      </c>
-      <c r="D954" t="s">
-        <v>2711</v>
       </c>
       <c r="E954" s="4" t="s">
         <v>721</v>
@@ -31985,13 +31985,13 @@
         <v>1845</v>
       </c>
       <c r="B961" t="s">
+        <v>2730</v>
+      </c>
+      <c r="C961" t="s">
+        <v>721</v>
+      </c>
+      <c r="D961" s="6" t="s">
         <v>2731</v>
-      </c>
-      <c r="C961" t="s">
-        <v>721</v>
-      </c>
-      <c r="D961" s="6" t="s">
-        <v>2732</v>
       </c>
       <c r="E961" s="4" t="s">
         <v>721</v>
@@ -32257,16 +32257,16 @@
     </row>
     <row r="975" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A975" t="s">
+        <v>2578</v>
+      </c>
+      <c r="B975" t="s">
         <v>2579</v>
       </c>
-      <c r="B975" t="s">
+      <c r="C975" t="s">
+        <v>721</v>
+      </c>
+      <c r="D975" s="6" t="s">
         <v>2580</v>
-      </c>
-      <c r="C975" t="s">
-        <v>721</v>
-      </c>
-      <c r="D975" s="6" t="s">
-        <v>2581</v>
       </c>
       <c r="E975" s="4" t="s">
         <v>721</v>
@@ -32280,10 +32280,10 @@
     </row>
     <row r="976" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A976" t="s">
+        <v>2611</v>
+      </c>
+      <c r="B976" t="s">
         <v>2612</v>
-      </c>
-      <c r="B976" t="s">
-        <v>2613</v>
       </c>
       <c r="C976" t="s">
         <v>721</v>
@@ -32306,10 +32306,10 @@
     </row>
     <row r="977" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A977" t="s">
+        <v>2613</v>
+      </c>
+      <c r="B977" t="s">
         <v>2614</v>
-      </c>
-      <c r="B977" t="s">
-        <v>2615</v>
       </c>
       <c r="C977" t="s">
         <v>721</v>
@@ -32332,16 +32332,16 @@
     </row>
     <row r="978" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A978" t="s">
+        <v>2615</v>
+      </c>
+      <c r="B978" t="s">
         <v>2616</v>
       </c>
-      <c r="B978" t="s">
+      <c r="C978" t="s">
+        <v>721</v>
+      </c>
+      <c r="D978" s="6" t="s">
         <v>2617</v>
-      </c>
-      <c r="C978" t="s">
-        <v>721</v>
-      </c>
-      <c r="D978" s="6" t="s">
-        <v>2618</v>
       </c>
       <c r="E978" s="4" t="s">
         <v>721</v>
@@ -32355,10 +32355,10 @@
     </row>
     <row r="979" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A979" t="s">
+        <v>2618</v>
+      </c>
+      <c r="B979" t="s">
         <v>2619</v>
-      </c>
-      <c r="B979" t="s">
-        <v>2620</v>
       </c>
       <c r="C979" t="s">
         <v>721</v>
@@ -32378,10 +32378,10 @@
     </row>
     <row r="980" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A980" t="s">
+        <v>2659</v>
+      </c>
+      <c r="B980" t="s">
         <v>2660</v>
-      </c>
-      <c r="B980" t="s">
-        <v>2661</v>
       </c>
       <c r="C980" t="s">
         <v>721</v>
@@ -32398,10 +32398,10 @@
     </row>
     <row r="981" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A981" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
       <c r="B981" t="s">
-        <v>2662</v>
+        <v>2661</v>
       </c>
       <c r="C981" t="s">
         <v>721</v>
@@ -32418,10 +32418,10 @@
     </row>
     <row r="982" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A982" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
       <c r="B982" t="s">
-        <v>2656</v>
+        <v>2655</v>
       </c>
       <c r="C982" t="s">
         <v>721</v>
@@ -32435,10 +32435,10 @@
     </row>
     <row r="983" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A983" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
       <c r="B983" t="s">
-        <v>2675</v>
+        <v>2674</v>
       </c>
       <c r="C983" t="s">
         <v>721</v>
@@ -32455,16 +32455,16 @@
     </row>
     <row r="984" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A984" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
       <c r="B984" t="s">
+        <v>2656</v>
+      </c>
+      <c r="C984" t="s">
+        <v>721</v>
+      </c>
+      <c r="D984" t="s">
         <v>2657</v>
-      </c>
-      <c r="C984" t="s">
-        <v>721</v>
-      </c>
-      <c r="D984" t="s">
-        <v>2658</v>
       </c>
       <c r="E984" s="4" t="s">
         <v>721</v>
@@ -32472,10 +32472,10 @@
     </row>
     <row r="985" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A985" t="s">
+        <v>2585</v>
+      </c>
+      <c r="B985" t="s">
         <v>2586</v>
-      </c>
-      <c r="B985" t="s">
-        <v>2587</v>
       </c>
       <c r="C985" t="s">
         <v>721</v>
@@ -32492,10 +32492,10 @@
     </row>
     <row r="986" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A986" t="s">
+        <v>2583</v>
+      </c>
+      <c r="B986" t="s">
         <v>2584</v>
-      </c>
-      <c r="B986" t="s">
-        <v>2585</v>
       </c>
       <c r="C986" t="s">
         <v>721</v>
@@ -32512,10 +32512,10 @@
     </row>
     <row r="987" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A987" t="s">
+        <v>2581</v>
+      </c>
+      <c r="B987" t="s">
         <v>2582</v>
-      </c>
-      <c r="B987" t="s">
-        <v>2583</v>
       </c>
       <c r="C987" t="s">
         <v>721</v>
@@ -32532,10 +32532,10 @@
     </row>
     <row r="988" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A988" t="s">
+        <v>2589</v>
+      </c>
+      <c r="B988" t="s">
         <v>2590</v>
-      </c>
-      <c r="B988" t="s">
-        <v>2591</v>
       </c>
       <c r="C988" t="s">
         <v>721</v>
@@ -32558,10 +32558,10 @@
     </row>
     <row r="989" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A989" t="s">
+        <v>2591</v>
+      </c>
+      <c r="B989" t="s">
         <v>2592</v>
-      </c>
-      <c r="B989" t="s">
-        <v>2593</v>
       </c>
       <c r="C989" t="s">
         <v>721</v>
@@ -32584,10 +32584,10 @@
     </row>
     <row r="990" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A990" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
       <c r="B990" t="s">
-        <v>2628</v>
+        <v>2627</v>
       </c>
       <c r="C990" t="s">
         <v>721</v>
@@ -32610,10 +32610,10 @@
     </row>
     <row r="991" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A991" t="s">
+        <v>2625</v>
+      </c>
+      <c r="B991" t="s">
         <v>2626</v>
-      </c>
-      <c r="B991" t="s">
-        <v>2627</v>
       </c>
       <c r="C991" t="s">
         <v>721</v>
@@ -32636,10 +32636,10 @@
     </row>
     <row r="992" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A992" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
       <c r="B992" t="s">
-        <v>2624</v>
+        <v>2623</v>
       </c>
       <c r="C992" t="s">
         <v>721</v>
@@ -32662,10 +32662,10 @@
     </row>
     <row r="993" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A993" t="s">
-        <v>2622</v>
+        <v>2621</v>
       </c>
       <c r="B993" t="s">
-        <v>2625</v>
+        <v>2624</v>
       </c>
       <c r="C993" t="s">
         <v>721</v>
@@ -32688,10 +32688,10 @@
     </row>
     <row r="994" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A994" t="s">
+        <v>2593</v>
+      </c>
+      <c r="B994" t="s">
         <v>2594</v>
-      </c>
-      <c r="B994" t="s">
-        <v>2595</v>
       </c>
       <c r="C994" t="s">
         <v>721</v>
@@ -32714,10 +32714,10 @@
     </row>
     <row r="995" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A995" t="s">
+        <v>2595</v>
+      </c>
+      <c r="B995" t="s">
         <v>2596</v>
-      </c>
-      <c r="B995" t="s">
-        <v>2597</v>
       </c>
       <c r="C995" t="s">
         <v>721</v>
@@ -32740,10 +32740,10 @@
     </row>
     <row r="996" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A996" t="s">
+        <v>2597</v>
+      </c>
+      <c r="B996" t="s">
         <v>2598</v>
-      </c>
-      <c r="B996" t="s">
-        <v>2599</v>
       </c>
       <c r="C996" t="s">
         <v>721</v>
@@ -32766,10 +32766,10 @@
     </row>
     <row r="997" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A997" t="s">
+        <v>2599</v>
+      </c>
+      <c r="B997" t="s">
         <v>2600</v>
-      </c>
-      <c r="B997" t="s">
-        <v>2601</v>
       </c>
       <c r="C997" t="s">
         <v>721</v>
@@ -32792,10 +32792,10 @@
     </row>
     <row r="998" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A998" t="s">
+        <v>2601</v>
+      </c>
+      <c r="B998" t="s">
         <v>2602</v>
-      </c>
-      <c r="B998" t="s">
-        <v>2603</v>
       </c>
       <c r="C998" t="s">
         <v>721</v>
@@ -32818,10 +32818,10 @@
     </row>
     <row r="999" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A999" t="s">
+        <v>2603</v>
+      </c>
+      <c r="B999" t="s">
         <v>2604</v>
-      </c>
-      <c r="B999" t="s">
-        <v>2605</v>
       </c>
       <c r="C999" t="s">
         <v>721</v>
@@ -32844,10 +32844,10 @@
     </row>
     <row r="1000" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1000" t="s">
+        <v>2605</v>
+      </c>
+      <c r="B1000" t="s">
         <v>2606</v>
-      </c>
-      <c r="B1000" t="s">
-        <v>2607</v>
       </c>
       <c r="C1000" t="s">
         <v>721</v>
@@ -32862,18 +32862,18 @@
         <v>1247</v>
       </c>
       <c r="H1000" s="3" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
       <c r="I1000" s="3" t="s">
-        <v>2659</v>
+        <v>2658</v>
       </c>
     </row>
     <row r="1001" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1001" t="s">
+        <v>2628</v>
+      </c>
+      <c r="B1001" t="s">
         <v>2629</v>
-      </c>
-      <c r="B1001" t="s">
-        <v>2630</v>
       </c>
       <c r="C1001" t="s">
         <v>721</v>
@@ -32896,10 +32896,10 @@
     </row>
     <row r="1002" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1002" t="s">
+        <v>2630</v>
+      </c>
+      <c r="B1002" t="s">
         <v>2631</v>
-      </c>
-      <c r="B1002" t="s">
-        <v>2632</v>
       </c>
       <c r="C1002" t="s">
         <v>721</v>
@@ -32916,16 +32916,16 @@
     </row>
     <row r="1003" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1003" t="s">
+        <v>2632</v>
+      </c>
+      <c r="B1003" t="s">
+        <v>2635</v>
+      </c>
+      <c r="C1003" t="s">
+        <v>721</v>
+      </c>
+      <c r="D1003" s="6" t="s">
         <v>2633</v>
-      </c>
-      <c r="B1003" t="s">
-        <v>2636</v>
-      </c>
-      <c r="C1003" t="s">
-        <v>721</v>
-      </c>
-      <c r="D1003" s="6" t="s">
-        <v>2634</v>
       </c>
       <c r="E1003" s="4" t="s">
         <v>721</v>
@@ -32939,10 +32939,10 @@
     </row>
     <row r="1004" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1004" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
       <c r="B1004" t="s">
-        <v>2637</v>
+        <v>2636</v>
       </c>
       <c r="C1004" t="s">
         <v>721</v>
@@ -32954,7 +32954,7 @@
         <v>142</v>
       </c>
       <c r="F1004" s="4" t="s">
-        <v>2638</v>
+        <v>2637</v>
       </c>
       <c r="H1004" s="2">
         <v>135</v>
@@ -32965,10 +32965,10 @@
     </row>
     <row r="1005" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1005" t="s">
+        <v>2638</v>
+      </c>
+      <c r="B1005" t="s">
         <v>2639</v>
-      </c>
-      <c r="B1005" t="s">
-        <v>2640</v>
       </c>
       <c r="C1005" t="s">
         <v>721</v>
@@ -32991,16 +32991,16 @@
     </row>
     <row r="1006" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1006" t="s">
+        <v>2640</v>
+      </c>
+      <c r="B1006" t="s">
         <v>2641</v>
       </c>
-      <c r="B1006" t="s">
-        <v>2642</v>
-      </c>
       <c r="C1006" t="s">
         <v>721</v>
       </c>
       <c r="D1006" s="6" t="s">
-        <v>2634</v>
+        <v>2633</v>
       </c>
       <c r="E1006" s="4" t="s">
         <v>721</v>
@@ -33014,16 +33014,16 @@
     </row>
     <row r="1007" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1007" t="s">
+        <v>2642</v>
+      </c>
+      <c r="B1007" t="s">
         <v>2643</v>
       </c>
-      <c r="B1007" t="s">
+      <c r="C1007" t="s">
+        <v>721</v>
+      </c>
+      <c r="D1007" s="6" t="s">
         <v>2644</v>
-      </c>
-      <c r="C1007" t="s">
-        <v>721</v>
-      </c>
-      <c r="D1007" s="6" t="s">
-        <v>2645</v>
       </c>
       <c r="E1007" s="4" t="s">
         <v>721</v>
@@ -33037,10 +33037,10 @@
     </row>
     <row r="1008" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1008" t="s">
+        <v>2645</v>
+      </c>
+      <c r="B1008" t="s">
         <v>2646</v>
-      </c>
-      <c r="B1008" t="s">
-        <v>2647</v>
       </c>
       <c r="C1008" t="s">
         <v>721</v>
@@ -33057,10 +33057,10 @@
     </row>
     <row r="1009" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1009" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
       <c r="B1009" t="s">
-        <v>2651</v>
+        <v>2650</v>
       </c>
       <c r="C1009" t="s">
         <v>721</v>
@@ -33077,10 +33077,10 @@
     </row>
     <row r="1010" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1010" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
       <c r="B1010" t="s">
-        <v>2652</v>
+        <v>2651</v>
       </c>
       <c r="C1010" t="s">
         <v>721</v>
@@ -33103,10 +33103,10 @@
     </row>
     <row r="1011" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1011" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
       <c r="B1011" t="s">
-        <v>2653</v>
+        <v>2652</v>
       </c>
       <c r="C1011" t="s">
         <v>721</v>
@@ -33131,10 +33131,10 @@
     </row>
     <row r="1013" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1013" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
       <c r="B1013" t="s">
-        <v>2683</v>
+        <v>2682</v>
       </c>
       <c r="C1013" t="s">
         <v>721</v>
@@ -33149,18 +33149,18 @@
         <v>1634</v>
       </c>
       <c r="H1013" s="2" t="s">
-        <v>2676</v>
+        <v>2675</v>
       </c>
       <c r="I1013" s="2" t="s">
-        <v>2676</v>
+        <v>2675</v>
       </c>
     </row>
     <row r="1014" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1014" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
       <c r="B1014" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1014" t="s">
         <v>721</v>
@@ -33175,18 +33175,18 @@
         <v>143</v>
       </c>
       <c r="H1014" s="2" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="I1014" s="2" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="1015" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1015" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
       <c r="B1015" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1015" t="s">
         <v>721</v>
@@ -33201,18 +33201,18 @@
         <v>143</v>
       </c>
       <c r="H1015" s="2" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
       <c r="I1015" s="2" t="s">
-        <v>2677</v>
+        <v>2676</v>
       </c>
     </row>
     <row r="1016" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1016" t="s">
-        <v>2688</v>
+        <v>2687</v>
       </c>
       <c r="B1016" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1016" t="s">
         <v>721</v>
@@ -33227,18 +33227,18 @@
         <v>143</v>
       </c>
       <c r="H1016" s="2" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="I1016" s="2" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
     </row>
     <row r="1017" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1017" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
       <c r="B1017" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1017" t="s">
         <v>721</v>
@@ -33253,18 +33253,18 @@
         <v>143</v>
       </c>
       <c r="H1017" s="2" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
       <c r="I1017" s="2" t="s">
-        <v>2678</v>
+        <v>2677</v>
       </c>
     </row>
     <row r="1018" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1018" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
       <c r="B1018" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1018" t="s">
         <v>721</v>
@@ -33279,18 +33279,18 @@
         <v>143</v>
       </c>
       <c r="H1018" s="2" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
       <c r="I1018" s="2" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="1019" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1019" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
       <c r="B1019" t="s">
-        <v>2684</v>
+        <v>2683</v>
       </c>
       <c r="C1019" t="s">
         <v>721</v>
@@ -33305,18 +33305,18 @@
         <v>143</v>
       </c>
       <c r="H1019" s="2" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
       <c r="I1019" s="2" t="s">
-        <v>2679</v>
+        <v>2678</v>
       </c>
     </row>
     <row r="1020" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1020" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
       <c r="B1020" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="C1020" t="s">
         <v>721</v>
@@ -33328,21 +33328,21 @@
         <v>1190</v>
       </c>
       <c r="F1020" s="4" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="H1020" s="2" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="I1020" s="2" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="1021" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1021" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
       <c r="B1021" t="s">
-        <v>2685</v>
+        <v>2684</v>
       </c>
       <c r="C1021" t="s">
         <v>721</v>
@@ -33354,21 +33354,21 @@
         <v>1190</v>
       </c>
       <c r="F1021" s="4" t="s">
-        <v>2608</v>
+        <v>2607</v>
       </c>
       <c r="H1021" s="2" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
       <c r="I1021" s="2" t="s">
-        <v>2680</v>
+        <v>2679</v>
       </c>
     </row>
     <row r="1022" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1022" t="s">
-        <v>2699</v>
+        <v>2698</v>
       </c>
       <c r="B1022" t="s">
-        <v>2610</v>
+        <v>2609</v>
       </c>
       <c r="C1022" t="s">
         <v>721</v>
@@ -33380,21 +33380,21 @@
         <v>1190</v>
       </c>
       <c r="F1022" s="4" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="H1022" s="3" t="s">
-        <v>2701</v>
+        <v>2700</v>
       </c>
       <c r="I1022" s="3" t="s">
-        <v>2701</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="1023" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1023" t="s">
-        <v>2700</v>
+        <v>2699</v>
       </c>
       <c r="B1023" t="s">
-        <v>2611</v>
+        <v>2610</v>
       </c>
       <c r="C1023" t="s">
         <v>721</v>
@@ -33406,27 +33406,27 @@
         <v>1190</v>
       </c>
       <c r="F1023" s="4" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="H1023" s="3" t="s">
-        <v>2702</v>
+        <v>2701</v>
       </c>
       <c r="I1023" s="3" t="s">
-        <v>2702</v>
+        <v>2701</v>
       </c>
     </row>
     <row r="1024" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1024" t="s">
-        <v>2697</v>
+        <v>2696</v>
       </c>
       <c r="B1024" t="s">
-        <v>2686</v>
+        <v>2685</v>
       </c>
       <c r="C1024" t="s">
         <v>721</v>
       </c>
       <c r="D1024" s="6" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="E1024" s="4" t="s">
         <v>142</v>
@@ -33435,24 +33435,24 @@
         <v>143</v>
       </c>
       <c r="H1024" s="2" t="s">
-        <v>2681</v>
+        <v>2680</v>
       </c>
       <c r="I1024" s="2" t="s">
-        <v>2681</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="1025" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1025" t="s">
-        <v>2698</v>
+        <v>2697</v>
       </c>
       <c r="B1025" t="s">
-        <v>2687</v>
+        <v>2686</v>
       </c>
       <c r="C1025" t="s">
         <v>721</v>
       </c>
       <c r="D1025" s="6" t="s">
-        <v>2609</v>
+        <v>2608</v>
       </c>
       <c r="E1025" s="4" t="s">
         <v>142</v>
@@ -33461,10 +33461,10 @@
         <v>143</v>
       </c>
       <c r="H1025" s="2" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
       <c r="I1025" s="2" t="s">
-        <v>2682</v>
+        <v>2681</v>
       </c>
     </row>
     <row r="1027" spans="1:9" x14ac:dyDescent="0.25">
@@ -33987,7 +33987,7 @@
         <v>721</v>
       </c>
       <c r="D1051" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="E1051" s="4" t="s">
         <v>721</v>
@@ -34015,10 +34015,10 @@
     </row>
     <row r="1053" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1053" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
       <c r="B1053" t="s">
-        <v>2577</v>
+        <v>2576</v>
       </c>
       <c r="C1053" t="s">
         <v>721</v>
@@ -34162,7 +34162,7 @@
         <v>721</v>
       </c>
       <c r="D1059" t="s">
-        <v>2575</v>
+        <v>2574</v>
       </c>
       <c r="E1059" s="4" t="s">
         <v>721</v>
@@ -34196,10 +34196,10 @@
     </row>
     <row r="1061" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1061" t="s">
+        <v>2575</v>
+      </c>
+      <c r="B1061" t="s">
         <v>2576</v>
-      </c>
-      <c r="B1061" t="s">
-        <v>2577</v>
       </c>
       <c r="C1061" t="s">
         <v>721</v>
@@ -35392,10 +35392,10 @@
     </row>
     <row r="1117" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1117" t="s">
+        <v>2458</v>
+      </c>
+      <c r="B1117" t="s">
         <v>2459</v>
-      </c>
-      <c r="B1117" t="s">
-        <v>2460</v>
       </c>
       <c r="C1117" t="s">
         <v>721</v>
@@ -35407,7 +35407,7 @@
         <v>1840</v>
       </c>
       <c r="F1117" s="4" t="s">
-        <v>2461</v>
+        <v>2460</v>
       </c>
       <c r="H1117" s="2">
         <v>60</v>
@@ -35444,10 +35444,10 @@
     </row>
     <row r="1119" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1119" t="s">
+        <v>2461</v>
+      </c>
+      <c r="B1119" t="s">
         <v>2462</v>
-      </c>
-      <c r="B1119" t="s">
-        <v>2463</v>
       </c>
       <c r="C1119" t="s">
         <v>721</v>
@@ -35459,7 +35459,7 @@
         <v>1840</v>
       </c>
       <c r="F1119" s="4" t="s">
-        <v>2464</v>
+        <v>2463</v>
       </c>
       <c r="H1119" s="2">
         <v>30</v>
@@ -35671,10 +35671,10 @@
     </row>
     <row r="1129" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1129" t="s">
+        <v>2572</v>
+      </c>
+      <c r="B1129" s="13" t="s">
         <v>2573</v>
-      </c>
-      <c r="B1129" s="13" t="s">
-        <v>2574</v>
       </c>
       <c r="C1129" t="s">
         <v>721</v>
@@ -36607,10 +36607,10 @@
     </row>
     <row r="1172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1172" t="s">
+        <v>2664</v>
+      </c>
+      <c r="B1172" t="s">
         <v>2665</v>
-      </c>
-      <c r="B1172" t="s">
-        <v>2666</v>
       </c>
       <c r="C1172" t="s">
         <v>721</v>
@@ -36913,10 +36913,10 @@
     </row>
     <row r="1190" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1190" t="s">
+        <v>2666</v>
+      </c>
+      <c r="B1190" t="s">
         <v>2667</v>
-      </c>
-      <c r="B1190" t="s">
-        <v>2668</v>
       </c>
       <c r="C1190" t="s">
         <v>721</v>
@@ -37628,7 +37628,7 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
-        <v>2543</v>
+        <v>2542</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.25">
@@ -37638,17 +37638,17 @@
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>2754</v>
+        <v>2753</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>2568</v>
+        <v>2567</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>2567</v>
+        <v>2566</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.25">
@@ -37663,142 +37663,142 @@
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>2669</v>
+        <v>2668</v>
       </c>
     </row>
     <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>2671</v>
+        <v>2670</v>
       </c>
     </row>
     <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>2703</v>
+        <v>2702</v>
       </c>
     </row>
     <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>2705</v>
+        <v>2704</v>
       </c>
     </row>
     <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>2564</v>
+        <v>2563</v>
       </c>
     </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>2713</v>
+        <v>2712</v>
       </c>
     </row>
     <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>2714</v>
+        <v>2713</v>
       </c>
     </row>
     <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>2715</v>
+        <v>2714</v>
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>2716</v>
+        <v>2715</v>
       </c>
     </row>
     <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>2717</v>
+        <v>2716</v>
       </c>
     </row>
     <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>2548</v>
+        <v>2547</v>
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>2546</v>
+        <v>2545</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>2550</v>
+        <v>2549</v>
       </c>
     </row>
     <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>2559</v>
+        <v>2558</v>
       </c>
     </row>
     <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>2563</v>
+        <v>2562</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>2723</v>
+        <v>2722</v>
       </c>
     </row>
     <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>2724</v>
+        <v>2723</v>
       </c>
     </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>2725</v>
+        <v>2724</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>2726</v>
+        <v>2725</v>
       </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>2736</v>
+        <v>2735</v>
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>2734</v>
+        <v>2733</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>2474</v>
+        <v>2473</v>
       </c>
     </row>
     <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>2471</v>
+        <v>2470</v>
       </c>
     </row>
     <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>2476</v>
+        <v>2475</v>
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>2478</v>
+        <v>2477</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>2480</v>
+        <v>2479</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>2481</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>2740</v>
+        <v>2739</v>
       </c>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.25">
@@ -37808,57 +37808,57 @@
     </row>
     <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>2508</v>
+        <v>2507</v>
       </c>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>2523</v>
+        <v>2522</v>
       </c>
     </row>
     <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>2525</v>
+        <v>2524</v>
       </c>
     </row>
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
-        <v>2510</v>
+        <v>2509</v>
       </c>
     </row>
     <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
-        <v>2521</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
-        <v>2539</v>
+        <v>2538</v>
       </c>
     </row>
     <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
-        <v>2513</v>
+        <v>2512</v>
       </c>
     </row>
     <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
-        <v>2516</v>
+        <v>2515</v>
       </c>
     </row>
     <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
-        <v>2519</v>
+        <v>2518</v>
       </c>
     </row>
     <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
-        <v>2520</v>
+        <v>2519</v>
       </c>
     </row>
     <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
-        <v>2487</v>
+        <v>2486</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
@@ -37873,12 +37873,12 @@
     </row>
     <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>2562</v>
+        <v>2561</v>
       </c>
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>2561</v>
+        <v>2560</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.25">
@@ -37898,42 +37898,42 @@
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>2495</v>
+        <v>2494</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>2498</v>
+        <v>2497</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>2499</v>
+        <v>2498</v>
       </c>
     </row>
     <row r="59" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>2500</v>
+        <v>2499</v>
       </c>
     </row>
     <row r="60" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
-        <v>2501</v>
+        <v>2500</v>
       </c>
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
-        <v>2502</v>
+        <v>2501</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
-        <v>2493</v>
+        <v>2492</v>
       </c>
     </row>
     <row r="63" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
-        <v>2491</v>
+        <v>2490</v>
       </c>
     </row>
     <row r="64" spans="1:1" x14ac:dyDescent="0.25">
@@ -37953,7 +37953,7 @@
     </row>
     <row r="67" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
-        <v>2571</v>
+        <v>2570</v>
       </c>
     </row>
     <row r="68" spans="1:1" x14ac:dyDescent="0.25">
@@ -38003,12 +38003,12 @@
     </row>
     <row r="77" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>2484</v>
+        <v>2483</v>
       </c>
     </row>
     <row r="78" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>2465</v>
+        <v>2464</v>
       </c>
     </row>
     <row r="79" spans="1:1" x14ac:dyDescent="0.25">
@@ -38023,302 +38023,302 @@
     </row>
     <row r="81" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>2733</v>
+        <v>2732</v>
       </c>
     </row>
     <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>2527</v>
+        <v>2526</v>
       </c>
     </row>
     <row r="83" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>2528</v>
+        <v>2527</v>
       </c>
     </row>
     <row r="84" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>2529</v>
+        <v>2528</v>
       </c>
     </row>
     <row r="85" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>2530</v>
+        <v>2529</v>
       </c>
     </row>
     <row r="86" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>2531</v>
+        <v>2530</v>
       </c>
     </row>
     <row r="87" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>2532</v>
+        <v>2531</v>
       </c>
     </row>
     <row r="88" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>2709</v>
+        <v>2708</v>
       </c>
     </row>
     <row r="89" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>2579</v>
+        <v>2578</v>
       </c>
     </row>
     <row r="90" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>2596</v>
+        <v>2595</v>
       </c>
     </row>
     <row r="91" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>2594</v>
+        <v>2593</v>
       </c>
     </row>
     <row r="92" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>2600</v>
+        <v>2599</v>
       </c>
     </row>
     <row r="93" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>2598</v>
+        <v>2597</v>
       </c>
     </row>
     <row r="94" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>2688</v>
+        <v>2687</v>
       </c>
     </row>
     <row r="95" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>2689</v>
+        <v>2688</v>
       </c>
     </row>
     <row r="96" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>2696</v>
+        <v>2695</v>
       </c>
     </row>
     <row r="97" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>2691</v>
+        <v>2690</v>
       </c>
     </row>
     <row r="98" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>2692</v>
+        <v>2691</v>
       </c>
     </row>
     <row r="99" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>2695</v>
+        <v>2694</v>
       </c>
     </row>
     <row r="100" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>2699</v>
+        <v>2698</v>
       </c>
     </row>
     <row r="101" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>2700</v>
+        <v>2699</v>
       </c>
     </row>
     <row r="102" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>2697</v>
+        <v>2696</v>
       </c>
     </row>
     <row r="103" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>2698</v>
+        <v>2697</v>
       </c>
     </row>
     <row r="104" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>2690</v>
+        <v>2689</v>
       </c>
     </row>
     <row r="105" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>2704</v>
+        <v>2703</v>
       </c>
     </row>
     <row r="106" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>2693</v>
+        <v>2692</v>
       </c>
     </row>
     <row r="107" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>2694</v>
+        <v>2693</v>
       </c>
     </row>
     <row r="108" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>2623</v>
+        <v>2622</v>
       </c>
     </row>
     <row r="109" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>2626</v>
+        <v>2625</v>
       </c>
     </row>
     <row r="110" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
-        <v>2612</v>
+        <v>2611</v>
       </c>
     </row>
     <row r="111" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
-        <v>2589</v>
+        <v>2588</v>
       </c>
     </row>
     <row r="112" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
-        <v>2654</v>
+        <v>2653</v>
       </c>
     </row>
     <row r="113" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
-        <v>2588</v>
+        <v>2587</v>
       </c>
     </row>
     <row r="114" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
-        <v>2655</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="115" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
-        <v>2586</v>
+        <v>2585</v>
       </c>
     </row>
     <row r="116" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
-        <v>2584</v>
+        <v>2583</v>
       </c>
     </row>
     <row r="117" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
-        <v>2582</v>
+        <v>2581</v>
       </c>
     </row>
     <row r="118" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
-        <v>2641</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="119" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
-        <v>2643</v>
+        <v>2642</v>
       </c>
     </row>
     <row r="120" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
-        <v>2648</v>
+        <v>2647</v>
       </c>
     </row>
     <row r="121" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
-        <v>2649</v>
+        <v>2648</v>
       </c>
     </row>
     <row r="122" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
-        <v>2650</v>
+        <v>2649</v>
       </c>
     </row>
     <row r="123" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
-        <v>2633</v>
+        <v>2632</v>
       </c>
     </row>
     <row r="124" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
-        <v>2635</v>
+        <v>2634</v>
       </c>
     </row>
     <row r="125" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
-        <v>2639</v>
+        <v>2638</v>
       </c>
     </row>
     <row r="126" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
-        <v>2646</v>
+        <v>2645</v>
       </c>
     </row>
     <row r="127" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
-        <v>2631</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="128" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
-        <v>2629</v>
+        <v>2628</v>
       </c>
     </row>
     <row r="129" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
-        <v>2614</v>
+        <v>2613</v>
       </c>
     </row>
     <row r="130" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
-        <v>2616</v>
+        <v>2615</v>
       </c>
     </row>
     <row r="131" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
-        <v>2619</v>
+        <v>2618</v>
       </c>
     </row>
     <row r="132" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
-        <v>2590</v>
+        <v>2589</v>
       </c>
     </row>
     <row r="133" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
-        <v>2592</v>
+        <v>2591</v>
       </c>
     </row>
     <row r="134" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
-        <v>2621</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="135" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
-        <v>2602</v>
+        <v>2601</v>
       </c>
     </row>
     <row r="136" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
-        <v>2604</v>
+        <v>2603</v>
       </c>
     </row>
     <row r="137" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
-        <v>2660</v>
+        <v>2659</v>
       </c>
     </row>
     <row r="138" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
-        <v>2606</v>
+        <v>2605</v>
       </c>
     </row>
     <row r="139" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
-        <v>2578</v>
+        <v>2577</v>
       </c>
     </row>
     <row r="140" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
-        <v>2576</v>
+        <v>2575</v>
       </c>
     </row>
     <row r="141" spans="1:1" x14ac:dyDescent="0.25">
@@ -38328,27 +38328,27 @@
     </row>
     <row r="142" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
-        <v>2462</v>
+        <v>2461</v>
       </c>
     </row>
     <row r="143" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
-        <v>2459</v>
+        <v>2458</v>
       </c>
     </row>
     <row r="144" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
-        <v>2573</v>
+        <v>2572</v>
       </c>
     </row>
     <row r="145" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
-        <v>2665</v>
+        <v>2664</v>
       </c>
     </row>
     <row r="146" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>2667</v>
+        <v>2666</v>
       </c>
     </row>
     <row r="149" spans="1:1" x14ac:dyDescent="0.25">
@@ -38457,340 +38457,340 @@
       <formula>H12&lt;&gt;I12</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A20 A23">
+    <cfRule type="expression" dxfId="465" priority="1540">
+      <formula>H6&lt;&gt;I6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A21 A32 A64 A83">
+    <cfRule type="expression" dxfId="464" priority="1584">
+      <formula>#REF!&lt;&gt;#REF!</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A22">
-    <cfRule type="expression" dxfId="465" priority="28">
+    <cfRule type="expression" dxfId="463" priority="28">
       <formula>H7&lt;&gt;I7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A23 A20">
-    <cfRule type="expression" dxfId="464" priority="1540">
-      <formula>H6&lt;&gt;I6</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A24:A28">
-    <cfRule type="expression" dxfId="463" priority="4">
+    <cfRule type="expression" dxfId="462" priority="4">
       <formula>H22&lt;&gt;I22</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A29">
-    <cfRule type="expression" dxfId="462" priority="6">
+    <cfRule type="expression" dxfId="461" priority="6">
       <formula>H26&lt;&gt;I26</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A33">
-    <cfRule type="expression" dxfId="461" priority="32">
-      <formula>H7&lt;&gt;I7</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A34 A31">
+  <conditionalFormatting sqref="A31 A34">
     <cfRule type="expression" dxfId="460" priority="1556">
       <formula>H6&lt;&gt;I6</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A33">
+    <cfRule type="expression" dxfId="459" priority="32">
+      <formula>H7&lt;&gt;I7</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A35 A38:A43">
-    <cfRule type="expression" dxfId="459" priority="38">
+    <cfRule type="expression" dxfId="458" priority="38">
       <formula>H8&lt;&gt;I8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A36">
-    <cfRule type="expression" dxfId="458" priority="3">
+    <cfRule type="expression" dxfId="457" priority="3">
       <formula>H34&lt;&gt;I34</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A37">
-    <cfRule type="expression" dxfId="457" priority="1504">
+    <cfRule type="expression" dxfId="456" priority="1504">
       <formula>H5&lt;&gt;I5</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A44:A47">
-    <cfRule type="expression" dxfId="456" priority="1496">
+    <cfRule type="expression" dxfId="455" priority="1496">
       <formula>H16&lt;&gt;I16</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A48">
-    <cfRule type="expression" dxfId="455" priority="1485">
+    <cfRule type="expression" dxfId="454" priority="1485">
       <formula>H11&lt;&gt;I11</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A49">
-    <cfRule type="expression" dxfId="454" priority="42">
+    <cfRule type="expression" dxfId="453" priority="42">
       <formula>H6&lt;&gt;I6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A50">
-    <cfRule type="expression" dxfId="453" priority="43">
+    <cfRule type="expression" dxfId="452" priority="43">
       <formula>H6&lt;&gt;I6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A51:A52">
-    <cfRule type="expression" dxfId="452" priority="29">
+    <cfRule type="expression" dxfId="451" priority="29">
       <formula>H28&lt;&gt;I28</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A53">
-    <cfRule type="expression" dxfId="451" priority="1513">
+    <cfRule type="expression" dxfId="450" priority="1513">
       <formula>H4&lt;&gt;I4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A55">
-    <cfRule type="expression" dxfId="450" priority="1483">
+    <cfRule type="expression" dxfId="449" priority="1483">
       <formula>H6&lt;&gt;I6</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A56">
-    <cfRule type="expression" dxfId="449" priority="1487">
+    <cfRule type="expression" dxfId="448" priority="1487">
       <formula>H15&lt;&gt;I15</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A57:A58">
-    <cfRule type="expression" dxfId="448" priority="1494">
+    <cfRule type="expression" dxfId="447" priority="1494">
       <formula>H12&lt;&gt;I12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A59:A63">
-    <cfRule type="expression" dxfId="447" priority="36">
+    <cfRule type="expression" dxfId="446" priority="36">
       <formula>H20&lt;&gt;I20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A65">
-    <cfRule type="expression" dxfId="446" priority="44">
+    <cfRule type="expression" dxfId="445" priority="44">
       <formula>H7&lt;&gt;I7</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A66 A73">
-    <cfRule type="expression" dxfId="445" priority="50">
+    <cfRule type="expression" dxfId="444" priority="50">
       <formula>H9&lt;&gt;I9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A67 A100 A104:A106">
-    <cfRule type="expression" dxfId="444" priority="24">
+    <cfRule type="expression" dxfId="443" priority="24">
       <formula>H49&lt;&gt;I49</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A68">
-    <cfRule type="expression" dxfId="443" priority="1515">
+    <cfRule type="expression" dxfId="442" priority="1515">
       <formula>H8&lt;&gt;I8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A69 A71">
-    <cfRule type="expression" dxfId="442" priority="1481">
+    <cfRule type="expression" dxfId="441" priority="1481">
       <formula>H4&lt;&gt;I4</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A72">
-    <cfRule type="expression" dxfId="441" priority="1489">
+    <cfRule type="expression" dxfId="440" priority="1489">
       <formula>H14&lt;&gt;I14</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A74:A75">
-    <cfRule type="expression" dxfId="440" priority="49">
+    <cfRule type="expression" dxfId="439" priority="49">
       <formula>H18&lt;&gt;I18</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A76">
-    <cfRule type="expression" dxfId="439" priority="1484">
+    <cfRule type="expression" dxfId="438" priority="1484">
       <formula>H23&lt;&gt;I23</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A77">
-    <cfRule type="expression" dxfId="438" priority="1499">
+    <cfRule type="expression" dxfId="437" priority="1499">
       <formula>H60&lt;&gt;I60</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A78">
-    <cfRule type="expression" dxfId="437" priority="39">
+    <cfRule type="expression" dxfId="436" priority="39">
       <formula>H20&lt;&gt;I20</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A79">
-    <cfRule type="expression" dxfId="436" priority="1495">
+    <cfRule type="expression" dxfId="435" priority="1495">
       <formula>H12&lt;&gt;I12</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A81">
-    <cfRule type="expression" dxfId="435" priority="9">
+    <cfRule type="expression" dxfId="434" priority="9">
       <formula>H76&lt;&gt;I76</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A87 A84">
-    <cfRule type="expression" dxfId="434" priority="1479">
+  <conditionalFormatting sqref="A82 A85">
+    <cfRule type="expression" dxfId="433" priority="1565">
+      <formula>H6&lt;&gt;I6</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A82:A87">
+    <cfRule type="expression" dxfId="432" priority="1498">
+      <formula>H20&lt;&gt;I20</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="A84 A87">
+    <cfRule type="expression" dxfId="431" priority="1479">
       <formula>H7&lt;&gt;I7</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="A82:A87">
-    <cfRule type="expression" dxfId="433" priority="1498">
-      <formula>H20&lt;&gt;I20</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A85 A82">
-    <cfRule type="expression" dxfId="432" priority="1565">
-      <formula>H6&lt;&gt;I6</formula>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="A86">
-    <cfRule type="expression" dxfId="431" priority="1551">
+    <cfRule type="expression" dxfId="430" priority="1551">
       <formula>H8&lt;&gt;I8</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A88">
-    <cfRule type="expression" dxfId="430" priority="13">
+    <cfRule type="expression" dxfId="429" priority="13">
       <formula>H73&lt;&gt;I73</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A89:A96 A103 A105 A145:A146">
-    <cfRule type="expression" dxfId="429" priority="16">
+    <cfRule type="expression" dxfId="428" priority="16">
       <formula>H69&lt;&gt;I69</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A94:A95">
-    <cfRule type="expression" dxfId="428" priority="1529">
+    <cfRule type="expression" dxfId="427" priority="1529">
       <formula>H108&lt;&gt;I108</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A96">
-    <cfRule type="expression" dxfId="427" priority="1547">
+    <cfRule type="expression" dxfId="426" priority="1547">
       <formula>H112&lt;&gt;I112</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="426" priority="1549">
+    <cfRule type="expression" dxfId="425" priority="1549">
       <formula>H113&lt;&gt;I113</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A97:A98 A101:A102">
-    <cfRule type="expression" dxfId="425" priority="1571">
+    <cfRule type="expression" dxfId="424" priority="1571">
       <formula>H110&lt;&gt;I110</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A97:A99">
-    <cfRule type="expression" dxfId="424" priority="1525">
+    <cfRule type="expression" dxfId="423" priority="1525">
       <formula>H111&lt;&gt;I111</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A99 A129 A135:A136 A138">
-    <cfRule type="expression" dxfId="423" priority="1575">
+    <cfRule type="expression" dxfId="422" priority="1575">
       <formula>H80&lt;&gt;I80</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A107">
-    <cfRule type="expression" dxfId="422" priority="1533">
+    <cfRule type="expression" dxfId="421" priority="1533">
       <formula>H118&lt;&gt;I118</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A108:A110">
-    <cfRule type="expression" dxfId="421" priority="1523">
+    <cfRule type="expression" dxfId="420" priority="1523">
       <formula>H74&lt;&gt;I74</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A111">
-    <cfRule type="expression" dxfId="420" priority="1581">
+    <cfRule type="expression" dxfId="419" priority="1581">
       <formula>H87&lt;&gt;I87</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A112:A128">
-    <cfRule type="expression" dxfId="419" priority="17">
+    <cfRule type="expression" dxfId="418" priority="17">
       <formula>H91&lt;&gt;I91</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A130:A131">
-    <cfRule type="expression" dxfId="418" priority="1526">
+    <cfRule type="expression" dxfId="417" priority="1526">
       <formula>H77&lt;&gt;I77</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A132">
-    <cfRule type="expression" dxfId="417" priority="1520">
+    <cfRule type="expression" dxfId="416" priority="1520">
       <formula>H81&lt;&gt;I81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A133">
-    <cfRule type="expression" dxfId="416" priority="1545">
+    <cfRule type="expression" dxfId="415" priority="1545">
       <formula>H79&lt;&gt;I79</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A134">
-    <cfRule type="expression" dxfId="415" priority="1538">
+    <cfRule type="expression" dxfId="414" priority="1538">
       <formula>H84&lt;&gt;I84</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A137">
-    <cfRule type="expression" dxfId="414" priority="1573">
+    <cfRule type="expression" dxfId="413" priority="1573">
       <formula>H88&lt;&gt;I88</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A139">
-    <cfRule type="expression" dxfId="413" priority="1541">
+    <cfRule type="expression" dxfId="412" priority="1541">
       <formula>H69&lt;&gt;I69</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A140">
-    <cfRule type="expression" dxfId="412" priority="1517">
+    <cfRule type="expression" dxfId="411" priority="1517">
       <formula>H87&lt;&gt;I87</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A141">
-    <cfRule type="expression" dxfId="411" priority="61">
+    <cfRule type="expression" dxfId="410" priority="61">
       <formula>H5&lt;&gt;I5</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="A142">
+    <cfRule type="expression" dxfId="409" priority="1594">
+      <formula>H26&lt;&gt;I26</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="408" priority="1595">
+      <formula>H4&lt;&gt;I4</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="A143">
-    <cfRule type="expression" dxfId="410" priority="41">
+    <cfRule type="expression" dxfId="407" priority="41">
       <formula>H25&lt;&gt;I25</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A144">
-    <cfRule type="expression" dxfId="409" priority="23">
+    <cfRule type="expression" dxfId="406" priority="23">
       <formula>H93&lt;&gt;I93</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A150">
-    <cfRule type="expression" dxfId="408" priority="10">
+    <cfRule type="expression" dxfId="405" priority="10">
       <formula>H144&lt;&gt;I144</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A151">
-    <cfRule type="expression" dxfId="407" priority="1516">
+    <cfRule type="expression" dxfId="404" priority="1516">
       <formula>H81&lt;&gt;I81</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A152">
-    <cfRule type="expression" dxfId="406" priority="1543">
+    <cfRule type="expression" dxfId="403" priority="1543">
       <formula>H79&lt;&gt;I79</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A156">
-    <cfRule type="expression" dxfId="405" priority="7">
+    <cfRule type="expression" dxfId="402" priority="7">
       <formula>H151&lt;&gt;I151</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A157">
-    <cfRule type="expression" dxfId="404" priority="5">
+    <cfRule type="expression" dxfId="401" priority="5">
       <formula>H153&lt;&gt;I153</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A158">
-    <cfRule type="expression" dxfId="403" priority="8">
+    <cfRule type="expression" dxfId="400" priority="8">
       <formula>H151&lt;&gt;I151</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A159:A163">
-    <cfRule type="expression" dxfId="402" priority="51">
+    <cfRule type="expression" dxfId="399" priority="51">
       <formula>H61&lt;&gt;I61</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A164">
-    <cfRule type="expression" dxfId="401" priority="1537">
+    <cfRule type="expression" dxfId="398" priority="1537">
       <formula>H86&lt;&gt;I86</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A21 A32 A64 A83">
-    <cfRule type="expression" dxfId="400" priority="1584">
-      <formula>#REF!&lt;&gt;#REF!</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="A142">
-    <cfRule type="expression" dxfId="399" priority="1594">
-      <formula>H26&lt;&gt;I26</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="398" priority="1595">
-      <formula>H4&lt;&gt;I4</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -41045,11 +41045,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A12">
-    <cfRule type="expression" dxfId="393" priority="798">
+    <cfRule type="expression" dxfId="393" priority="803">
+      <formula>F9&lt;&gt;G9</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="392" priority="798">
       <formula>F6&lt;&gt;G6</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="392" priority="803">
-      <formula>F9&lt;&gt;G9</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A13">
@@ -41755,11 +41755,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A243">
-    <cfRule type="expression" dxfId="249" priority="1283">
+    <cfRule type="expression" dxfId="249" priority="1284">
+      <formula>F109&lt;&gt;G109</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="248" priority="1283">
       <formula>F41&lt;&gt;G41</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="248" priority="1284">
-      <formula>F109&lt;&gt;G109</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A244">
@@ -41793,11 +41793,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A250">
-    <cfRule type="expression" dxfId="241" priority="961">
+    <cfRule type="expression" dxfId="241" priority="1031">
+      <formula>F75&lt;&gt;G75</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="240" priority="961">
       <formula>F59&lt;&gt;G59</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="240" priority="1031">
-      <formula>F75&lt;&gt;G75</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A251">
@@ -41848,11 +41848,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A258">
-    <cfRule type="expression" dxfId="228" priority="1288">
+    <cfRule type="expression" dxfId="228" priority="1289">
+      <formula>F43&lt;&gt;G43</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="227" priority="1288">
       <formula>F63&lt;&gt;G63</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="227" priority="1289">
-      <formula>F43&lt;&gt;G43</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A259">
@@ -42209,11 +42209,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A380:A389">
-    <cfRule type="expression" dxfId="155" priority="131">
+    <cfRule type="expression" dxfId="155" priority="993">
+      <formula>F56&lt;&gt;G56</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="154" priority="131">
       <formula>F197&lt;&gt;G197</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="154" priority="993">
-      <formula>F56&lt;&gt;G56</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A385">
@@ -42272,11 +42272,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A404">
-    <cfRule type="expression" dxfId="142" priority="1377">
+    <cfRule type="expression" dxfId="142" priority="1378">
+      <formula>F36&lt;&gt;G36</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="141" priority="1377">
       <formula>F243&lt;&gt;G243</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="141" priority="1378">
-      <formula>F36&lt;&gt;G36</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A405">

</xml_diff>